<commit_message>
Account ad Excel Chnages
</commit_message>
<xml_diff>
--- a/src/modules/Masters/AccountsManagement/CustomerAccountCreation/data/CustomerAccountCreation.xlsx
+++ b/src/modules/Masters/AccountsManagement/CustomerAccountCreation/data/CustomerAccountCreation.xlsx
@@ -9,109 +9,176 @@
     <sheet sheetId="3" name="Authorize" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="Negative" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="Database" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="AuthorizedList" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="52">
+  <si>
+    <t>testTag</t>
+  </si>
+  <si>
+    <t>customerNumber</t>
+  </si>
+  <si>
+    <t>moduleCode</t>
+  </si>
+  <si>
+    <t>productCode</t>
+  </si>
+  <si>
+    <t>schemeCode</t>
+  </si>
+  <si>
+    <t>modeOfOperation</t>
+  </si>
+  <si>
+    <t>nomineeYN</t>
+  </si>
+  <si>
+    <t>stmtFreq</t>
+  </si>
+  <si>
+    <t>stmtMode</t>
+  </si>
+  <si>
+    <t>@sanity</t>
+  </si>
+  <si>
+    <t>1395042</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>15101</t>
+  </si>
+  <si>
+    <t>01</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>@regression</t>
+  </si>
+  <si>
+    <t>accountNo</t>
+  </si>
+  <si>
+    <t>authStatus</t>
+  </si>
+  <si>
+    <t>createdAt</t>
+  </si>
+  <si>
+    <t>scenario</t>
+  </si>
+  <si>
+    <t>expectedError</t>
+  </si>
+  <si>
+    <t>Empty customerNumber</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>15201</t>
+  </si>
+  <si>
+    <t>Save confirm modal</t>
+  </si>
+  <si>
+    <t>Empty moduleCode</t>
+  </si>
+  <si>
+    <t>Empty form</t>
+  </si>
   <si>
     <t>customerId</t>
   </si>
   <si>
-    <t>accountType</t>
-  </si>
-  <si>
-    <t>branchCode</t>
-  </si>
-  <si>
-    <t>initialDeposit</t>
-  </si>
-  <si>
-    <t>nomineeName</t>
-  </si>
-  <si>
-    <t>nomineeRelation</t>
-  </si>
-  <si>
-    <t>CUST001</t>
-  </si>
-  <si>
-    <t>SAVINGS</t>
-  </si>
-  <si>
-    <t>001</t>
-  </si>
-  <si>
-    <t>10000</t>
-  </si>
-  <si>
-    <t>Spouse Name</t>
-  </si>
-  <si>
-    <t>SPOUSE</t>
-  </si>
-  <si>
-    <t>CUST002</t>
-  </si>
-  <si>
-    <t>CURRENT</t>
-  </si>
-  <si>
-    <t>25000</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>accountNumber</t>
-  </si>
-  <si>
-    <t>ACC001</t>
-  </si>
-  <si>
-    <t>New Nominee</t>
-  </si>
-  <si>
-    <t>PARENT</t>
-  </si>
-  <si>
     <t>expectedStatus</t>
   </si>
   <si>
-    <t>AUTHORIZED</t>
-  </si>
-  <si>
-    <t>scenario</t>
-  </si>
-  <si>
-    <t>expectedError</t>
-  </si>
-  <si>
-    <t>Invalid Customer</t>
-  </si>
-  <si>
-    <t>INVALID999</t>
-  </si>
-  <si>
-    <t>Zero Deposit</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>expectedType</t>
-  </si>
-  <si>
-    <t>ACTIVE</t>
+    <t>expectedModuleCode</t>
+  </si>
+  <si>
+    <t>authorizedAt</t>
+  </si>
+  <si>
+    <t>139015201755557</t>
+  </si>
+  <si>
+    <t>Authorized</t>
+  </si>
+  <si>
+    <t>27/8/2026, 8:52:31 am</t>
+  </si>
+  <si>
+    <t>139015201755553</t>
+  </si>
+  <si>
+    <t>27/8/2026, 8:52:43 am</t>
+  </si>
+  <si>
+    <t>139015201755554</t>
+  </si>
+  <si>
+    <t>27/8/2026, 8:52:56 am</t>
+  </si>
+  <si>
+    <t>139015201755555</t>
+  </si>
+  <si>
+    <t>27/8/2026, 8:53:09 am</t>
+  </si>
+  <si>
+    <t>139015201755556</t>
+  </si>
+  <si>
+    <t>27/8/2026, 8:53:22 am</t>
+  </si>
+  <si>
+    <t>139015101001320</t>
+  </si>
+  <si>
+    <t>27/8/2026, 9:08:39 am</t>
+  </si>
+  <si>
+    <t>139015101001321</t>
+  </si>
+  <si>
+    <t>27/8/2026, 9:09:01 am</t>
+  </si>
+  <si>
+    <t>139015101001322</t>
+  </si>
+  <si>
+    <t>27/8/2026, 9:09:21 am</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -119,13 +186,22 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4472C4"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -140,8 +216,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -481,226 +558,512 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="9" width="20" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+      <c r="G2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="6" width="20" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" t="s">
-        <v>19</v>
+      <c r="D1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="7" width="20" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="G1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="7" width="20" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>25</v>
       </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="E2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>3</v>
+        <v>25</v>
+      </c>
+      <c r="F3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="5" width="20" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>29</v>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="7" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" t="s">
+        <v>36</v>
+      </c>
+      <c r="G8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" t="s">
+        <v>36</v>
+      </c>
+      <c r="G9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>